<commit_message>
đổi trạng thái, sửa luồng đối soát file mẫu hoá đơn
</commit_message>
<xml_diff>
--- a/public/templates/MAU_XUAT-HD.xlsx
+++ b/public/templates/MAU_XUAT-HD.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>CÔNG TY TNHH HÓA ĐƠN ĐIỆN TỬ M-INVOICE - CN TP. HỒ CHÍ MINH</t>
   </si>
@@ -44,13 +44,13 @@
     <t xml:space="preserve">BẢNG ĐỐI SOÁT ĐẠI LÝ: </t>
   </si>
   <si>
-    <t>THÁNG 1/2026</t>
+    <t>THÁNG</t>
   </si>
   <si>
     <t>STT</t>
   </si>
   <si>
-    <t>THÁNG PHÁT SINH</t>
+    <t>NGÀY PHÁT SINH</t>
   </si>
   <si>
     <t>MÃ SỐ THUẾ</t>
@@ -62,7 +62,7 @@
     <t>LOẠI SP</t>
   </si>
   <si>
-    <t>GÓI CƯỚC PHẦN MỀM</t>
+    <t>SỐ LƯỢNG</t>
   </si>
   <si>
     <t>DT KHÁC</t>
@@ -87,15 +87,6 @@
     <t>GHI CHÚ</t>
   </si>
   <si>
-    <t>BẢN QUYỀN</t>
-  </si>
-  <si>
-    <t>SỐ LƯỢNG</t>
-  </si>
-  <si>
-    <t>GÓI HÓA ĐƠN</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
@@ -123,7 +114,7 @@
     <t>GIÁ TRỊ THANH TOÁN ( âm ( M-invoice chi) và dương  ( M-invoice thu)</t>
   </si>
   <si>
-    <t>HCM, ngày 04 tháng 3 năm 2026</t>
+    <t xml:space="preserve">HCM, ngày  tháng  năm </t>
   </si>
   <si>
     <t>Xác nhận đại lý</t>
@@ -136,8 +127,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="8">
-    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+  <numFmts count="7">
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
@@ -146,7 +136,7 @@
     <numFmt numFmtId="178" formatCode="_-* #,##0.00\ _₫_-;\-* #,##0.00\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
     <numFmt numFmtId="179" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="34">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,13 +191,15 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
     <font>
+      <i/>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
@@ -225,13 +217,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <i/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -595,7 +580,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -641,21 +626,6 @@
       <top/>
       <bottom style="thin">
         <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -814,144 +784,144 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="178" fontId="32" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="33" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="178" fontId="34" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="178" fontId="32" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="178" fontId="31" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -960,11 +930,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -973,9 +943,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -983,6 +950,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1010,26 +980,30 @@
     <xf numFmtId="179" fontId="7" fillId="0" borderId="1" xfId="52" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="179" fontId="7" fillId="0" borderId="1" xfId="53" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="179" fontId="7" fillId="0" borderId="1" xfId="52" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="179" fontId="2" fillId="3" borderId="1" xfId="54" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="55" applyFont="1" applyAlignment="1">
@@ -1038,41 +1012,37 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="179" fontId="7" fillId="0" borderId="1" xfId="52" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="179" fontId="7" fillId="0" borderId="1" xfId="53" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="179" fontId="7" fillId="0" borderId="1" xfId="52" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="179" fontId="2" fillId="0" borderId="1" xfId="54" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="179" fontId="1" fillId="0" borderId="1" xfId="54" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="179" fontId="11" fillId="0" borderId="1" xfId="54" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="179" fontId="9" fillId="0" borderId="1" xfId="54" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="8" fillId="0" borderId="1" xfId="54" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="179" fontId="9" fillId="0" borderId="1" xfId="52" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="179" fontId="8" fillId="0" borderId="1" xfId="52" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="51" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="179" fontId="2" fillId="0" borderId="0" xfId="54" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1080,10 +1050,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="179" fontId="7" fillId="0" borderId="0" xfId="52" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="49" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="49" applyFont="1"/>
   </cellXfs>
   <cellStyles count="56">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1422,6 +1389,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>107950</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>80010</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="833986" cy="597941"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="107950" y="80010"/>
+          <a:ext cx="833755" cy="597535"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1683,7 +1694,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Q22"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultColWidth="8.05555555555556" defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="5.27777777777778" style="2" customWidth="1"/>
@@ -1692,108 +1703,95 @@
     <col min="4" max="4" width="45.9722222222222" style="2" customWidth="1"/>
     <col min="5" max="5" width="9.30555555555556" style="2" customWidth="1"/>
     <col min="6" max="6" width="11.8055555555556" style="2" customWidth="1"/>
-    <col min="7" max="7" width="9.72222222222222" style="2" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="11.25" style="2" customWidth="1"/>
-    <col min="10" max="10" width="11.3888888888889" style="2" customWidth="1"/>
-    <col min="11" max="11" width="10.1388888888889" style="2" customWidth="1"/>
-    <col min="12" max="12" width="12.6388888888889" style="2" customWidth="1"/>
-    <col min="13" max="13" width="16.6666666666667" style="2" customWidth="1"/>
-    <col min="14" max="14" width="10.5555555555556" style="2" customWidth="1"/>
-    <col min="15" max="15" width="9.30555555555556" style="2" customWidth="1"/>
-    <col min="16" max="17" width="8.75" style="2" customWidth="1"/>
-    <col min="18" max="16384" width="8.05555555555556" style="2"/>
+    <col min="7" max="7" width="11.25" style="2" customWidth="1"/>
+    <col min="8" max="8" width="11.3888888888889" style="2" customWidth="1"/>
+    <col min="9" max="9" width="10.1388888888889" style="2" customWidth="1"/>
+    <col min="10" max="10" width="12.6388888888889" style="2" customWidth="1"/>
+    <col min="11" max="11" width="16.6666666666667" style="2" customWidth="1"/>
+    <col min="12" max="12" width="10.5555555555556" style="2" customWidth="1"/>
+    <col min="13" max="13" width="9.30555555555556" style="2" customWidth="1"/>
+    <col min="14" max="15" width="8.75" style="2" customWidth="1"/>
+    <col min="16" max="16384" width="8.05555555555556" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="23.45" customHeight="1" spans="3:10">
+    <row r="1" s="1" customFormat="1" ht="23.45" customHeight="1" spans="3:8">
       <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="4"/>
-      <c r="J1" s="3"/>
-    </row>
-    <row r="2" s="1" customFormat="1" ht="23.45" customHeight="1" spans="3:9">
-      <c r="C2" s="5" t="s">
+      <c r="H1" s="3"/>
+    </row>
+    <row r="2" s="1" customFormat="1" ht="23.45" customHeight="1" spans="3:7">
+      <c r="C2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="3"/>
-      <c r="I2" s="33"/>
-    </row>
-    <row r="3" s="1" customFormat="1" ht="23.45" customHeight="1" spans="3:9">
-      <c r="C3" s="5" t="s">
+      <c r="G2" s="5"/>
+    </row>
+    <row r="3" s="1" customFormat="1" ht="23.45" customHeight="1" spans="3:7">
+      <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="3"/>
-    </row>
-    <row r="4" s="1" customFormat="1" ht="23.45" customHeight="1" spans="1:9">
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" s="1" customFormat="1" ht="23.45" customHeight="1" spans="1:7">
       <c r="A4" s="6"/>
       <c r="B4" s="7"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="8"/>
-    </row>
-    <row r="5" s="1" customFormat="1" ht="23.45" customHeight="1" spans="1:15">
-      <c r="A5" s="10" t="s">
+    </row>
+    <row r="5" s="1" customFormat="1" ht="23.45" customHeight="1" spans="1:13">
+      <c r="A5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10"/>
-      <c r="O5" s="10"/>
-    </row>
-    <row r="6" s="1" customFormat="1" ht="23.45" customHeight="1" spans="1:15">
-      <c r="A6" s="11" t="s">
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" s="1" customFormat="1" ht="23.45" customHeight="1" spans="1:13">
+      <c r="A6" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-    </row>
-    <row r="7" s="1" customFormat="1" ht="23.45" customHeight="1" spans="1:15">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7"/>
-      <c r="F7"/>
-      <c r="G7"/>
-      <c r="H7"/>
-      <c r="I7"/>
-      <c r="J7"/>
-      <c r="K7"/>
-      <c r="L7"/>
-      <c r="M7"/>
-      <c r="N7"/>
-      <c r="O7"/>
-    </row>
-    <row r="8" s="2" customFormat="1" ht="21" customHeight="1" spans="1:15">
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+    </row>
+    <row r="7" s="1" customFormat="1" ht="23.45" customHeight="1" spans="1:13">
+      <c r="A7" s="11"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
+    </row>
+    <row r="8" s="2" customFormat="1" ht="21" customHeight="1" spans="1:13">
       <c r="A8" s="13" t="s">
         <v>5</v>
       </c>
@@ -1809,135 +1807,106 @@
       <c r="E8" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
+      <c r="G8" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="13" t="s">
+        <v>12</v>
+      </c>
       <c r="I8" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="J8" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="K8" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="L8" s="34" t="s">
+      <c r="J8" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="M8" s="34" t="s">
+      <c r="K8" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="N8" s="34" t="s">
+      <c r="L8" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="13" t="s">
+      <c r="M8" s="13" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" s="2" customFormat="1" ht="31" customHeight="1" spans="1:15">
+    <row r="9" s="2" customFormat="1" ht="31" customHeight="1" spans="1:13">
       <c r="A9" s="13"/>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="15"/>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="15"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="38"/>
+      <c r="K9" s="38"/>
+      <c r="L9" s="38"/>
+      <c r="M9" s="13"/>
+    </row>
+    <row r="10" s="2" customFormat="1" spans="1:13">
+      <c r="A10" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="B10" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="C10" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="35"/>
-      <c r="M9" s="35"/>
-      <c r="N9" s="35"/>
-      <c r="O9" s="13"/>
-    </row>
-    <row r="10" s="2" customFormat="1" spans="1:15">
-      <c r="A10" s="16" t="s">
+      <c r="D10" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>24</v>
-      </c>
       <c r="E10" s="16"/>
-      <c r="F10" s="16">
-        <v>1</v>
-      </c>
+      <c r="F10" s="16"/>
       <c r="G10" s="16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H10" s="16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I10" s="16">
-        <v>4</v>
-      </c>
-      <c r="J10" s="16">
-        <v>5</v>
-      </c>
-      <c r="K10" s="16">
         <v>6</v>
       </c>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
       <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="16"/>
-      <c r="O10" s="16">
+      <c r="M10" s="16">
         <v>7</v>
       </c>
     </row>
-    <row r="11" s="2" customFormat="1" ht="27" customHeight="1" spans="1:15">
+    <row r="11" s="2" customFormat="1" ht="27" customHeight="1" spans="1:13">
       <c r="A11" s="17"/>
       <c r="B11" s="18"/>
       <c r="C11" s="19"/>
       <c r="D11" s="20"/>
       <c r="E11" s="21"/>
-      <c r="F11" s="22"/>
+      <c r="F11" s="21"/>
       <c r="G11" s="22"/>
       <c r="H11" s="23"/>
-      <c r="I11" s="36"/>
-      <c r="J11" s="37">
-        <f>F11+H11+I11</f>
+      <c r="I11" s="23">
+        <f>H11-J11</f>
         <v>0</v>
       </c>
-      <c r="K11" s="37"/>
-      <c r="L11" s="23">
-        <f>J11-K11</f>
-        <v>0</v>
-      </c>
-      <c r="M11" s="23"/>
-      <c r="N11" s="23">
-        <f>J11-M11</f>
-        <v>0</v>
-      </c>
-      <c r="O11" s="38"/>
-    </row>
-    <row r="12" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:15">
+      <c r="J11" s="39"/>
+      <c r="K11" s="39"/>
+      <c r="L11" s="39"/>
+      <c r="M11" s="40"/>
+    </row>
+    <row r="12" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:13">
       <c r="A12" s="24" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B12" s="24"/>
       <c r="C12" s="24"/>
       <c r="D12" s="24"/>
       <c r="E12" s="24"/>
-      <c r="F12" s="25">
-        <f t="shared" ref="F12:N12" si="0">SUM(F11:F11)</f>
-        <v>0</v>
-      </c>
+      <c r="F12" s="24"/>
       <c r="G12" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="G12:L12" si="0">SUM(G11:G11)</f>
         <v>0</v>
       </c>
       <c r="H12" s="25">
@@ -1960,19 +1929,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M12" s="25">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="N12" s="25">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O12" s="25"/>
-    </row>
-    <row r="13" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:17">
+      <c r="M12" s="25"/>
+    </row>
+    <row r="13" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:15">
       <c r="A13" s="26" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B13" s="27"/>
       <c r="C13" s="27"/>
@@ -1980,22 +1941,21 @@
       <c r="E13" s="27"/>
       <c r="F13" s="27"/>
       <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="39"/>
-      <c r="K13" s="40">
-        <f>K12</f>
+      <c r="H13" s="28"/>
+      <c r="I13" s="41">
+        <f>I12</f>
         <v>0</v>
       </c>
-      <c r="L13" s="40"/>
-      <c r="M13" s="40"/>
-      <c r="N13" s="41"/>
-      <c r="O13" s="37"/>
-      <c r="Q13" s="42"/>
-    </row>
-    <row r="14" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:16">
+      <c r="J13" s="41"/>
+      <c r="K13" s="41"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="23"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="36"/>
+    </row>
+    <row r="14" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:13">
       <c r="A14" s="26" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B14" s="27"/>
       <c r="C14" s="27"/>
@@ -2003,22 +1963,19 @@
       <c r="E14" s="27"/>
       <c r="F14" s="27"/>
       <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="39"/>
-      <c r="K14" s="40"/>
-      <c r="L14" s="40"/>
-      <c r="M14" s="40">
-        <f>M12</f>
+      <c r="H14" s="28"/>
+      <c r="I14" s="41"/>
+      <c r="J14" s="41"/>
+      <c r="K14" s="41">
+        <f>K12</f>
         <v>0</v>
       </c>
-      <c r="N14" s="40"/>
-      <c r="O14" s="37"/>
-      <c r="P14" s="42"/>
-    </row>
-    <row r="15" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:15">
+      <c r="L14" s="41"/>
+      <c r="M14" s="23"/>
+    </row>
+    <row r="15" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:13">
       <c r="A15" s="26" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B15" s="27"/>
       <c r="C15" s="27"/>
@@ -2026,121 +1983,112 @@
       <c r="E15" s="27"/>
       <c r="F15" s="27"/>
       <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="39"/>
-      <c r="K15" s="40"/>
-      <c r="L15" s="40">
-        <f>L12</f>
+      <c r="H15" s="28"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41">
+        <f>J12</f>
         <v>0</v>
       </c>
-      <c r="M15" s="40"/>
-      <c r="N15" s="41"/>
-      <c r="O15" s="37"/>
-    </row>
-    <row r="16" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:15">
-      <c r="A16" s="28" t="s">
+      <c r="K15" s="41"/>
+      <c r="L15" s="42"/>
+      <c r="M15" s="23"/>
+    </row>
+    <row r="16" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:14">
+      <c r="A16" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="43"/>
+      <c r="J16" s="43"/>
+      <c r="K16" s="43">
+        <f>H12-J12-K12</f>
+        <v>0</v>
+      </c>
+      <c r="L16" s="44"/>
+      <c r="M16" s="45"/>
+      <c r="N16" s="46"/>
+    </row>
+    <row r="17" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:13">
+      <c r="A17" s="32"/>
+      <c r="B17" s="32"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="47"/>
+      <c r="J17" s="47"/>
+      <c r="K17" s="47"/>
+      <c r="L17" s="48"/>
+      <c r="M17" s="49"/>
+    </row>
+    <row r="18" s="1" customFormat="1" spans="2:13">
+      <c r="B18" s="7"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="H18" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="I18" s="50"/>
+      <c r="J18" s="50"/>
+      <c r="K18" s="50"/>
+      <c r="L18" s="50"/>
+      <c r="M18" s="50"/>
+    </row>
+    <row r="19" s="1" customFormat="1" ht="16.9" customHeight="1" spans="3:8">
+      <c r="C19" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="H19" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="29"/>
-      <c r="H16" s="29"/>
-      <c r="I16" s="29"/>
-      <c r="J16" s="43"/>
-      <c r="K16" s="44"/>
-      <c r="L16" s="44"/>
-      <c r="M16" s="44">
-        <f>J12-L12-M12</f>
-        <v>0</v>
-      </c>
-      <c r="N16" s="45"/>
-      <c r="O16" s="46"/>
-    </row>
-    <row r="17" s="2" customFormat="1" ht="19.35" customHeight="1" spans="1:15">
-      <c r="A17" s="30"/>
-      <c r="B17" s="30"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-      <c r="I17" s="30"/>
-      <c r="J17" s="30"/>
-      <c r="K17" s="47"/>
-      <c r="L17" s="47"/>
-      <c r="M17" s="47"/>
-      <c r="N17" s="48"/>
-      <c r="O17" s="49"/>
-    </row>
-    <row r="18" s="1" customFormat="1" spans="2:15">
-      <c r="B18" s="7"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="J18" s="50" t="s">
-        <v>30</v>
-      </c>
-      <c r="K18" s="51"/>
-      <c r="L18" s="51"/>
-      <c r="M18" s="51"/>
-      <c r="N18" s="51"/>
-      <c r="O18" s="51"/>
-    </row>
-    <row r="19" s="1" customFormat="1" ht="16.9" customHeight="1" spans="3:10">
-      <c r="C19" s="31" t="s">
-        <v>31</v>
-      </c>
-      <c r="J19" s="31" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="20" s="1" customFormat="1" spans="2:7">
+    </row>
+    <row r="20" s="1" customFormat="1" spans="2:2">
       <c r="B20" s="7"/>
-      <c r="G20" s="7"/>
-    </row>
-    <row r="21" s="1" customFormat="1" spans="2:9">
+    </row>
+    <row r="21" s="1" customFormat="1" spans="2:7">
       <c r="B21" s="7"/>
-      <c r="F21" s="32"/>
+      <c r="F21" s="35"/>
       <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-    </row>
-    <row r="22" s="2" customFormat="1" spans="6:10">
-      <c r="F22" s="32"/>
-      <c r="J22" s="42"/>
+    </row>
+    <row r="22" s="2" customFormat="1" spans="6:8">
+      <c r="F22" s="35"/>
+      <c r="H22" s="36"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="F8:H8"/>
+  <mergeCells count="22">
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A6:M6"/>
     <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="A14:J14"/>
-    <mergeCell ref="A15:J15"/>
-    <mergeCell ref="A16:J16"/>
-    <mergeCell ref="J18:O18"/>
-    <mergeCell ref="J19:O19"/>
-    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="H18:M18"/>
+    <mergeCell ref="H19:M19"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="D8:D9"/>
     <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
     <mergeCell ref="I8:I9"/>
     <mergeCell ref="J8:J9"/>
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="L8:L9"/>
     <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="O8:O9"/>
   </mergeCells>
   <conditionalFormatting sqref="D11">
-    <cfRule type="duplicateValues" dxfId="0" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>